<commit_message>
feat: Add detailed documentation for SFA business flows, code mapping, and offline architecture
- Created SFA-BUSINESS-FLOWS.md to outline comprehensive business processes for field sales, order placement, customer check-in/out, inventory tasks, and offline synchronization.
- Introduced SFA-CODE-MAP.md for quick reference to file locations corresponding to business functionalities within the Flutter mobile application.
- Added SFA-OFFLINE-ARCH.md detailing the offline architecture, state management rules, sync processes, and conflict detection mechanisms.
</commit_message>
<xml_diff>
--- a/output/IMPORT_SAN_PHAM.xlsx
+++ b/output/IMPORT_SAN_PHAM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\HQSOFT\PROJECTS\CUSTOM\Xspire_AVN\ai-skills\output\2026-06-26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\HQSOFT\PROJECTS\CUSTOM\Xspire_AVN\ai-skills\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56FC8398-F9C7-43DF-B840-8313BD100A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ACADC50-3251-410C-92A6-56B737C662FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{314DB58B-7B90-45B8-810C-3378FE83243B}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{314DB58B-7B90-45B8-810C-3378FE83243B}"/>
   </bookViews>
   <sheets>
     <sheet name="Products" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="112">
   <si>
     <t>Mã khách hàng</t>
   </si>
@@ -295,43 +295,73 @@
     <t>ChangeID</t>
   </si>
   <si>
-    <t>Bag AN Pork 900g-campaign (06.23)</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
     <t>FEFO</t>
   </si>
   <si>
-    <t>Z006</t>
-  </si>
-  <si>
     <t>U</t>
   </si>
   <si>
-    <t>PCS</t>
-  </si>
-  <si>
-    <t>Carton AN Pork 170g - Jar AZ01 (10.19)</t>
-  </si>
-  <si>
-    <t>CARTON AN PORK 170G - JAR AZ01 (10.19)</t>
-  </si>
-  <si>
-    <t>Thùng AN Heo 170g - Hủ AZ01</t>
-  </si>
-  <si>
-    <t>Bag AN Pork and Shrimp 2kg (04.23)</t>
-  </si>
-  <si>
     <t>AVN</t>
   </si>
   <si>
-    <t>CB</t>
-  </si>
-  <si>
-    <t>PAL</t>
+    <t>M-400G-L-TET-(10.20)</t>
+  </si>
+  <si>
+    <t>AJI-NO-MOTO 400gL15</t>
+  </si>
+  <si>
+    <t>Bột ngọt AJI-NO-MOTO 400gL15</t>
+  </si>
+  <si>
+    <t>BAG, CAS</t>
+  </si>
+  <si>
+    <t>CAS</t>
+  </si>
+  <si>
+    <t>Z002</t>
+  </si>
+  <si>
+    <t>KG</t>
+  </si>
+  <si>
+    <t>AN-50G-CHICKEN-(09.20)</t>
+  </si>
+  <si>
+    <t>Aji-ngon gà 50g1</t>
+  </si>
+  <si>
+    <t>Hạt nêm Aji-ngon 50gG1</t>
+  </si>
+  <si>
+    <t>BAG, INN, CAS</t>
+  </si>
+  <si>
+    <t>M-400G-L-(10.20)</t>
+  </si>
+  <si>
+    <t>AJI-NO-MOTO 400gL14 test rút gọn</t>
+  </si>
+  <si>
+    <t>Bột ngọt AJI-NO-MOTO 400gL14 test tên trên hóa đơn</t>
+  </si>
+  <si>
+    <t>HỘP QUÀ TẾT 2023 SUM VẦY</t>
+  </si>
+  <si>
+    <t>BOX, CAS</t>
+  </si>
+  <si>
+    <t>Z013</t>
+  </si>
+  <si>
+    <t>BOX</t>
+  </si>
+  <si>
+    <t>BAG</t>
   </si>
 </sst>
 </file>
@@ -395,12 +425,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -715,7 +746,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDC864B0-CEDA-4E4A-8796-7D97EC1E7407}">
-  <dimension ref="A1:AI5"/>
+  <dimension ref="A1:AI6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="24" width="14.77734375" customWidth="1"/>
@@ -939,52 +970,79 @@
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>142003912</v>
+        <v>140002608</v>
       </c>
       <c r="B3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D3" t="s">
         <v>89</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="b">
+        <v>0</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>0.4</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3" t="s">
         <v>90</v>
       </c>
-      <c r="E3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3" t="b">
-        <v>0</v>
-      </c>
-      <c r="G3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
+        <v>95</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>101</v>
+      </c>
+      <c r="N3">
+        <v>102</v>
+      </c>
+      <c r="O3">
+        <v>999999</v>
+      </c>
+      <c r="P3">
+        <v>19</v>
+      </c>
+      <c r="Q3" t="b">
+        <v>0</v>
+      </c>
+      <c r="R3" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>97</v>
+      </c>
+      <c r="AC3" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE3" t="s">
         <v>91</v>
       </c>
-      <c r="Q3" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z3">
-        <v>0</v>
-      </c>
-      <c r="AA3">
-        <v>0</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>92</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>93</v>
+      <c r="AF3" t="s">
+        <v>95</v>
       </c>
       <c r="AG3">
         <v>1</v>
       </c>
       <c r="AH3" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="AI3" t="b">
         <v>0</v>
@@ -992,61 +1050,79 @@
     </row>
     <row r="4" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>142002875</v>
+        <v>140002579</v>
       </c>
       <c r="B4" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C4" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+      <c r="F4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>0.05</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4" t="s">
         <v>90</v>
       </c>
-      <c r="E4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F4" t="b">
-        <v>0</v>
-      </c>
-      <c r="G4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
+        <v>102</v>
+      </c>
+      <c r="L4">
+        <v>2</v>
+      </c>
+      <c r="M4">
+        <v>201</v>
+      </c>
+      <c r="N4">
+        <v>100</v>
+      </c>
+      <c r="O4">
+        <v>20103</v>
+      </c>
+      <c r="P4">
+        <v>7</v>
+      </c>
+      <c r="Q4" t="b">
+        <v>0</v>
+      </c>
+      <c r="R4" t="s">
+        <v>103</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>97</v>
+      </c>
+      <c r="AC4" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="AD4" t="s">
+        <v>98</v>
+      </c>
+      <c r="AE4" t="s">
         <v>91</v>
       </c>
-      <c r="K4" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q4" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z4">
-        <v>0</v>
-      </c>
-      <c r="AA4">
-        <v>0</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>92</v>
-      </c>
-      <c r="AE4" t="s">
-        <v>93</v>
-      </c>
       <c r="AF4" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="AG4">
         <v>1</v>
       </c>
       <c r="AH4" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="AI4" t="b">
         <v>0</v>
@@ -1054,55 +1130,147 @@
     </row>
     <row r="5" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>142003876</v>
+        <v>140002583</v>
       </c>
       <c r="B5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>0.4</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5" t="s">
+        <v>90</v>
+      </c>
+      <c r="K5" t="s">
+        <v>106</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>101</v>
+      </c>
+      <c r="N5">
+        <v>102</v>
+      </c>
+      <c r="O5">
+        <v>999999</v>
+      </c>
+      <c r="P5">
+        <v>19</v>
+      </c>
+      <c r="Q5" t="b">
+        <v>0</v>
+      </c>
+      <c r="R5" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>97</v>
+      </c>
+      <c r="AC5" s="3">
+        <v>0.4</v>
+      </c>
+      <c r="AD5" t="s">
         <v>98</v>
       </c>
-      <c r="D5" t="s">
+      <c r="AE5" t="s">
+        <v>91</v>
+      </c>
+      <c r="AF5" t="s">
+        <v>106</v>
+      </c>
+      <c r="AG5">
+        <v>1</v>
+      </c>
+      <c r="AH5" t="s">
+        <v>99</v>
+      </c>
+      <c r="AI5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:35" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>140002773</v>
+      </c>
+      <c r="B6" t="s">
+        <v>107</v>
+      </c>
+      <c r="C6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D6" t="s">
+        <v>89</v>
+      </c>
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1.21</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6" t="s">
         <v>90</v>
       </c>
-      <c r="E5" t="b">
-        <v>1</v>
-      </c>
-      <c r="F5" t="b">
-        <v>0</v>
-      </c>
-      <c r="G5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5" t="s">
+      <c r="K6" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q6" t="b">
+        <v>0</v>
+      </c>
+      <c r="R6" t="s">
+        <v>108</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>97</v>
+      </c>
+      <c r="AC6">
+        <v>1.21</v>
+      </c>
+      <c r="AD6" t="s">
+        <v>109</v>
+      </c>
+      <c r="AE6" t="s">
         <v>91</v>
       </c>
-      <c r="Q5" t="b">
-        <v>0</v>
-      </c>
-      <c r="Z5">
-        <v>0</v>
-      </c>
-      <c r="AA5">
-        <v>0</v>
-      </c>
-      <c r="AD5" t="s">
-        <v>92</v>
-      </c>
-      <c r="AE5" t="s">
-        <v>93</v>
-      </c>
-      <c r="AG5">
-        <v>1</v>
-      </c>
-      <c r="AH5" t="s">
-        <v>94</v>
-      </c>
-      <c r="AI5" t="b">
-        <v>0</v>
+      <c r="AF6" t="s">
+        <v>107</v>
+      </c>
+      <c r="AG6">
+        <v>1</v>
+      </c>
+      <c r="AH6" t="s">
+        <v>110</v>
+      </c>
+      <c r="AI6" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1112,7 +1280,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4794A66-BA9E-43E0-B93C-BBEBBE4ED1E1}">
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="3" width="14.77734375" customWidth="1"/>
@@ -1199,116 +1367,344 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>691.2</v>
+        <v>1</v>
       </c>
       <c r="B3">
-        <v>799.12800000000004</v>
+        <v>1.06</v>
       </c>
       <c r="C3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H3">
+        <v>140002608</v>
+      </c>
+      <c r="I3" t="s">
         <v>99</v>
       </c>
-      <c r="H3">
-        <v>140003227</v>
-      </c>
-      <c r="I3" t="s">
-        <v>100</v>
-      </c>
       <c r="J3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3">
-        <v>1000</v>
+        <v>2500</v>
       </c>
       <c r="L3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="B4">
-        <v>0</v>
+        <v>12.724</v>
       </c>
       <c r="C4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D4">
         <v>12</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="H4">
-        <v>142002344</v>
+        <v>140002608</v>
       </c>
       <c r="I4" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="J4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>30000</v>
       </c>
       <c r="L4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>529.20000000000005</v>
+        <v>0.4</v>
       </c>
       <c r="B5">
-        <v>575.1</v>
+        <v>0.40799999999999997</v>
       </c>
       <c r="C5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5">
-        <v>529.20000000000005</v>
+        <v>0.4</v>
       </c>
       <c r="E5">
-        <v>108</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5" t="s">
+        <v>92</v>
+      </c>
+      <c r="H5">
+        <v>140002608</v>
+      </c>
+      <c r="I5" t="s">
+        <v>111</v>
+      </c>
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>1000</v>
+      </c>
+      <c r="L5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6">
+        <v>1.133</v>
+      </c>
+      <c r="C6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>20</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6" t="s">
+        <v>92</v>
+      </c>
+      <c r="H6">
+        <v>140002579</v>
+      </c>
+      <c r="I6" t="s">
         <v>99</v>
       </c>
-      <c r="H5">
-        <v>140001127</v>
-      </c>
-      <c r="I5" t="s">
-        <v>101</v>
-      </c>
-      <c r="J5" t="b">
-        <v>0</v>
-      </c>
-      <c r="K5">
-        <v>108000</v>
-      </c>
-      <c r="L5" t="s">
-        <v>93</v>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>20000</v>
+      </c>
+      <c r="L6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>7.5</v>
+      </c>
+      <c r="B7">
+        <v>8.4979999999999993</v>
+      </c>
+      <c r="C7" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>7.5</v>
+      </c>
+      <c r="E7">
+        <v>150</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>92</v>
+      </c>
+      <c r="H7">
+        <v>140002579</v>
+      </c>
+      <c r="I7" t="s">
+        <v>97</v>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7">
+        <v>150000</v>
+      </c>
+      <c r="L7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>0.05</v>
+      </c>
+      <c r="B8">
+        <v>5.2999999999999999E-2</v>
+      </c>
+      <c r="C8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8">
+        <v>0.05</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>3</v>
+      </c>
+      <c r="G8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H8">
+        <v>140002579</v>
+      </c>
+      <c r="I8" t="s">
+        <v>111</v>
+      </c>
+      <c r="J8" t="b">
+        <v>1</v>
+      </c>
+      <c r="K8">
+        <v>1000</v>
+      </c>
+      <c r="L8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>0.999</v>
+      </c>
+      <c r="B9">
+        <v>1.089</v>
+      </c>
+      <c r="C9" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0.82599999999999996</v>
+      </c>
+      <c r="E9">
+        <v>0.82599999999999996</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H9">
+        <v>140002773</v>
+      </c>
+      <c r="I9" t="s">
+        <v>99</v>
+      </c>
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>826</v>
+      </c>
+      <c r="L9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>7.26</v>
+      </c>
+      <c r="B10">
+        <v>8.5579999999999998</v>
+      </c>
+      <c r="C10" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>6</v>
+      </c>
+      <c r="E10">
+        <v>6</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>92</v>
+      </c>
+      <c r="H10">
+        <v>140002773</v>
+      </c>
+      <c r="I10" t="s">
+        <v>97</v>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10">
+        <v>6000</v>
+      </c>
+      <c r="L10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1.21</v>
+      </c>
+      <c r="B11">
+        <v>1.3180000000000001</v>
+      </c>
+      <c r="C11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>2</v>
+      </c>
+      <c r="G11" t="s">
+        <v>92</v>
+      </c>
+      <c r="H11">
+        <v>140002773</v>
+      </c>
+      <c r="I11" t="s">
+        <v>110</v>
+      </c>
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
+      <c r="K11">
+        <v>1000</v>
+      </c>
+      <c r="L11" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>